<commit_message>
feat(parrillero-2.2): F2 cerrada — los 11 entregables 2.2 en dl/ y gates D15 en verde
Motor TODO VERDE, calculadora 552/552, 112 arreglos de texto + A4 en los otros 7, docx 11 H1 / 8.120 palabras,
censo 0 defectos, no latinos 0. Mac = VPS byte a byte.

Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/plan-negocio-parrillero-asador-eventos/plantilla-proveedores-parrillero-asador-eventos.xlsx
+++ b/astro-site/public/dl/plan-negocio-parrillero-asador-eventos/plantilla-proveedores-parrillero-asador-eventos.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Carniceria mayorista" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Carbon, leña y combustible" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Equipamiento parrilla y asad" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Cuchilleria, tablas, menaje " sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Cuchilleria, tablas, menaje" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Vajilla, cuberteria, mantele" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Indumentaria y proteccion" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Seguros, gestoria y asesoria" sheetId="8" state="visible" r:id="rId8"/>
@@ -23,7 +23,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'1. Carniceria mayorista'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'2. Carbon, leña y combustible'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'3. Equipamiento parrilla y asad'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'4. Cuchilleria, tablas, menaje '!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'4. Cuchilleria, tablas, menaje'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'5. Vajilla, cuberteria, mantele'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'6. Indumentaria y proteccion'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'7. Seguros, gestoria y asesoria'!$4:$4</definedName>
@@ -124,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -140,6 +140,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -518,18 +521,17 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plantilla 96 Proveedores · Parrillero / Asador para Eventos</t>
+          <t>Plantilla de 93 proveedores · Parrillero / Asador para Eventos</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Listado vivo. Marca como [validado] solo cuando hayas trabajado con el proveedor o tengas referencias directas. Score 1-10 segun tu experiencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Listado vivo. «Por verificar» significa que aún no has trabajado con el proveedor ni tienes referencias directas: pasa a «Contactado» u «Homologado» cuando las tengas. El score de 1 a 10 lo pones tú según tu experiencia.</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -578,7 +580,11 @@
       <c r="C6" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="D6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Ver la nota EUDR al final de la hoja</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="4" t="n">
@@ -704,11 +710,10 @@
       </c>
       <c r="D15" s="4" t="inlineStr"/>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Versión 1.1 · agosto 2026 · aichef.pro/plan-negocio-parrillero-asador-eventos · info@aichef.pro</t>
+          <t>Versión 2.2 · octubre 2026 · aichef.pro/plan-negocio-parrillero-asador-eventos · info@aichef.pro</t>
         </is>
       </c>
     </row>
@@ -834,14 +839,10 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>10/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Critico</t>
@@ -876,14 +877,10 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
@@ -914,14 +911,10 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
@@ -952,14 +945,10 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="24" customHeight="1">
@@ -990,14 +979,10 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -1028,14 +1013,10 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="24" customHeight="1">
@@ -1066,14 +1047,10 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="24" customHeight="1">
@@ -1104,14 +1081,10 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="24" customHeight="1">
@@ -1142,14 +1115,10 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="24" customHeight="1">
@@ -1180,14 +1149,10 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="n"/>
       <c r="H14" s="5" t="inlineStr">
         <is>
           <t>Stand o pase visitante</t>
@@ -1199,6 +1164,11 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F5:F14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Por verificar,Contactado,Homologado,Investigar"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -1316,14 +1286,10 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>10/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Acceso 360+ proveedores</t>
@@ -1358,14 +1324,10 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
@@ -1396,14 +1358,10 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
@@ -1434,14 +1392,10 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="inlineStr"/>
     </row>
   </sheetData>
@@ -1449,6 +1403,11 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F5:F8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Por verificar,Contactado,Homologado,Investigar"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -1566,14 +1525,10 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="24" customHeight="1">
@@ -1604,14 +1559,10 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
@@ -1642,14 +1593,10 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Premium para B2B</t>
@@ -1684,14 +1631,10 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="24" customHeight="1">
@@ -1722,14 +1665,10 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -1760,14 +1699,10 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="24" customHeight="1">
@@ -1798,14 +1733,10 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="24" customHeight="1">
@@ -1836,14 +1767,10 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="24" customHeight="1">
@@ -1874,14 +1801,10 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="24" customHeight="1">
@@ -1912,14 +1835,10 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="n"/>
       <c r="H14" s="5" t="inlineStr"/>
     </row>
     <row r="15" ht="24" customHeight="1">
@@ -1950,14 +1869,10 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="n"/>
       <c r="H15" s="4" t="inlineStr"/>
     </row>
     <row r="16" ht="24" customHeight="1">
@@ -1988,14 +1903,10 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="n"/>
       <c r="H16" s="5" t="inlineStr"/>
     </row>
   </sheetData>
@@ -2003,6 +1914,11 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F5:F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Por verificar,Contactado,Homologado,Investigar"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -2022,7 +1938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2120,14 +2036,10 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Hostelero</t>
@@ -2162,14 +2074,10 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
@@ -2200,14 +2108,10 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
@@ -2238,14 +2142,10 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="24" customHeight="1">
@@ -2276,14 +2176,10 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -2314,14 +2210,10 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="24" customHeight="1">
@@ -2352,14 +2244,10 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="24" customHeight="1">
@@ -2390,14 +2278,10 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>6/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="24" customHeight="1">
@@ -2428,21 +2312,30 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="inlineStr"/>
     </row>
+    <row r="15" ht="62" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Nota EUDR: si tu carbón o tu leña son de marabú (Cuba, África) o de quebracho (Paraguay, Argentina) importados, pueden ser madera afectada por el Reglamento (UE) 2023/1115 (EUDR). La obligación recae en el importador desde el 30-12-2026 (empresas grandes y medianas) o el 30-06-2027 (micro y pequeñas): pide a tu proveedor la declaración de diligencia debida.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A15:H15"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F5:F13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Por verificar,Contactado,Homologado,Investigar"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -2560,14 +2453,10 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>10/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Proveedor referencia</t>
@@ -2602,14 +2491,10 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
@@ -2640,14 +2525,10 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
@@ -2678,14 +2559,10 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="24" customHeight="1">
@@ -2716,14 +2593,10 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -2754,14 +2627,10 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="24" customHeight="1">
@@ -2792,14 +2661,10 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Para BBQ texano</t>
@@ -2834,14 +2699,10 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="inlineStr">
         <is>
           <t>Concepto pizzero</t>
@@ -2876,14 +2737,10 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="24" customHeight="1">
@@ -2914,14 +2771,10 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>6/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="n"/>
       <c r="H14" s="5" t="inlineStr"/>
     </row>
     <row r="15" ht="24" customHeight="1">
@@ -2952,14 +2805,10 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="n"/>
       <c r="H15" s="4" t="inlineStr"/>
     </row>
     <row r="16" ht="24" customHeight="1">
@@ -2990,14 +2839,10 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="n"/>
       <c r="H16" s="5" t="inlineStr"/>
     </row>
     <row r="17" ht="24" customHeight="1">
@@ -3028,14 +2873,10 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>6/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="n"/>
       <c r="H17" s="4" t="inlineStr"/>
     </row>
   </sheetData>
@@ -3043,6 +2884,11 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F5:F17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Por verificar,Contactado,Homologado,Investigar"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -3160,14 +3006,10 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>10/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Marca lider España</t>
@@ -3202,14 +3044,10 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
@@ -3240,14 +3078,10 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
@@ -3278,14 +3112,10 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="24" customHeight="1">
@@ -3316,14 +3146,10 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -3354,14 +3180,10 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="24" customHeight="1">
@@ -3392,14 +3214,10 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="24" customHeight="1">
@@ -3430,14 +3248,10 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="24" customHeight="1">
@@ -3468,14 +3282,10 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="inlineStr"/>
     </row>
   </sheetData>
@@ -3483,6 +3293,11 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F5:F13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Por verificar,Contactado,Homologado,Investigar"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -3600,14 +3415,10 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Eco-friendly</t>
@@ -3642,14 +3453,10 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
@@ -3680,14 +3487,10 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
@@ -3718,14 +3521,10 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="24" customHeight="1">
@@ -3756,14 +3555,10 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -3794,14 +3589,10 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="24" customHeight="1">
@@ -3832,14 +3623,10 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="24" customHeight="1">
@@ -3870,14 +3657,10 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>6/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="24" customHeight="1">
@@ -3908,14 +3691,10 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Sostenible</t>
@@ -3950,14 +3729,10 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="n"/>
       <c r="H14" s="5" t="inlineStr"/>
     </row>
   </sheetData>
@@ -3965,6 +3740,11 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F5:F14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Por verificar,Contactado,Homologado,Investigar"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -4082,14 +3862,10 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>10/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>EPI certificado</t>
@@ -4124,14 +3900,10 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
@@ -4162,14 +3934,10 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
@@ -4200,14 +3968,10 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>6/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="24" customHeight="1">
@@ -4238,14 +4002,10 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -4276,14 +4036,10 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="inlineStr">
         <is>
           <t>Linea premium</t>
@@ -4318,14 +4074,10 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="24" customHeight="1">
@@ -4356,14 +4108,10 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>6/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="inlineStr"/>
     </row>
   </sheetData>
@@ -4371,6 +4119,11 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F5:F12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Por verificar,Contactado,Homologado,Investigar"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -4488,14 +4241,10 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Recomendado planners</t>
@@ -4530,14 +4279,10 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
@@ -4568,14 +4313,10 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
@@ -4606,14 +4347,10 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="24" customHeight="1">
@@ -4644,14 +4381,10 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -4682,14 +4415,10 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="24" customHeight="1">
@@ -4720,14 +4449,10 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="24" customHeight="1">
@@ -4758,14 +4483,10 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="24" customHeight="1">
@@ -4796,14 +4517,10 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="24" customHeight="1">
@@ -4834,14 +4551,10 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>6/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="n"/>
       <c r="H14" s="5" t="inlineStr"/>
     </row>
   </sheetData>
@@ -4849,6 +4562,11 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F5:F14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Por verificar,Contactado,Homologado,Investigar"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -4966,14 +4684,10 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Escalado food truck</t>
@@ -5008,14 +4722,10 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
@@ -5046,14 +4756,10 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>8/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="24" customHeight="1">
@@ -5084,14 +4790,10 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>validado</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="24" customHeight="1">
@@ -5122,14 +4824,10 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -5160,14 +4858,10 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="24" customHeight="1">
@@ -5198,14 +4892,10 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>6/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="24" customHeight="1">
@@ -5236,14 +4926,10 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>investigar</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>7/10</t>
-        </is>
-      </c>
+          <t>Investigar</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="inlineStr"/>
     </row>
   </sheetData>
@@ -5251,6 +4937,11 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F5:F12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Por verificar,Contactado,Homologado,Investigar"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>

</xml_diff>